<commit_message>
Reset Excel Table for Crane no.2
</commit_message>
<xml_diff>
--- a/FM-MN-07_Crane no.2.xlsx
+++ b/FM-MN-07_Crane no.2.xlsx
@@ -1776,11 +1776,7 @@
           <t>ตรวจเช็คปุ่มกดต้องอยู่ในสภาพพร้อมใช้งาน ไม่แตก ไม่ชำรุด เสียหาย</t>
         </is>
       </c>
-      <c r="C6" s="29" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C6" s="29" t="inlineStr"/>
       <c r="D6" s="29" t="inlineStr"/>
       <c r="E6" s="29" t="inlineStr"/>
       <c r="F6" s="29" t="inlineStr"/>
@@ -1821,11 +1817,7 @@
           <t>ตรวจเช็คการหยุดเครน เดินหน้า และถอยหลัง เมื่อปล่อยปุ่มกดต้องหยุดทันที</t>
         </is>
       </c>
-      <c r="C7" s="29" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C7" s="29" t="inlineStr"/>
       <c r="D7" s="29" t="inlineStr"/>
       <c r="E7" s="29" t="inlineStr"/>
       <c r="F7" s="29" t="inlineStr"/>
@@ -1867,11 +1859,7 @@
 และบิดงอ</t>
         </is>
       </c>
-      <c r="C8" s="29" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C8" s="29" t="inlineStr"/>
       <c r="D8" s="29" t="inlineStr"/>
       <c r="E8" s="29" t="inlineStr"/>
       <c r="F8" s="29" t="inlineStr"/>
@@ -1912,11 +1900,7 @@
           <t>ตรวจเช็คตะขอต้องไม่มีรอยแตกร้าวสูญหายกิ๊ปปากตะขอไม่ชำรุดหรือหลุดหาย</t>
         </is>
       </c>
-      <c r="C9" s="29" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C9" s="29" t="inlineStr"/>
       <c r="D9" s="29" t="inlineStr"/>
       <c r="E9" s="29" t="inlineStr"/>
       <c r="F9" s="29" t="inlineStr"/>
@@ -1958,11 +1942,7 @@
 ไม่เรียบร้อย</t>
         </is>
       </c>
-      <c r="C10" s="29" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C10" s="29" t="inlineStr"/>
       <c r="D10" s="29" t="inlineStr"/>
       <c r="E10" s="29" t="inlineStr"/>
       <c r="F10" s="29" t="inlineStr"/>
@@ -2003,11 +1983,7 @@
           <t>ตรวจเช็คสัญญานเสียงเมื่อเริ่มเดินเครนต้องมีเสียงเตือนการทำงาน</t>
         </is>
       </c>
-      <c r="C11" s="29" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C11" s="29" t="inlineStr"/>
       <c r="D11" s="29" t="inlineStr"/>
       <c r="E11" s="29" t="inlineStr"/>
       <c r="F11" s="29" t="inlineStr"/>
@@ -2110,11 +2086,7 @@
     <row r="14" ht="22.5" customHeight="1">
       <c r="A14" s="11" t="n"/>
       <c r="B14" s="10" t="n"/>
-      <c r="C14" s="46" t="inlineStr">
-        <is>
-          <t>นพดล สุระแสน</t>
-        </is>
-      </c>
+      <c r="C14" s="46" t="inlineStr"/>
       <c r="D14" s="44" t="inlineStr"/>
       <c r="E14" s="44" t="inlineStr"/>
       <c r="F14" s="44" t="inlineStr"/>

</xml_diff>

<commit_message>
Direct Write Excel for Crane no.2 Day 6
</commit_message>
<xml_diff>
--- a/FM-MN-07_Crane no.2.xlsx
+++ b/FM-MN-07_Crane no.2.xlsx
@@ -1781,7 +1781,11 @@
       <c r="E6" s="29" t="inlineStr"/>
       <c r="F6" s="29" t="inlineStr"/>
       <c r="G6" s="29" t="inlineStr"/>
-      <c r="H6" s="29" t="inlineStr"/>
+      <c r="H6" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I6" s="29" t="inlineStr"/>
       <c r="J6" s="29" t="inlineStr"/>
       <c r="K6" s="29" t="inlineStr"/>
@@ -1822,7 +1826,11 @@
       <c r="E7" s="29" t="inlineStr"/>
       <c r="F7" s="29" t="inlineStr"/>
       <c r="G7" s="29" t="inlineStr"/>
-      <c r="H7" s="29" t="inlineStr"/>
+      <c r="H7" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I7" s="29" t="inlineStr"/>
       <c r="J7" s="29" t="inlineStr"/>
       <c r="K7" s="29" t="inlineStr"/>
@@ -1864,7 +1872,11 @@
       <c r="E8" s="29" t="inlineStr"/>
       <c r="F8" s="29" t="inlineStr"/>
       <c r="G8" s="29" t="inlineStr"/>
-      <c r="H8" s="29" t="inlineStr"/>
+      <c r="H8" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I8" s="29" t="inlineStr"/>
       <c r="J8" s="29" t="inlineStr"/>
       <c r="K8" s="29" t="inlineStr"/>
@@ -1905,7 +1917,11 @@
       <c r="E9" s="29" t="inlineStr"/>
       <c r="F9" s="29" t="inlineStr"/>
       <c r="G9" s="29" t="inlineStr"/>
-      <c r="H9" s="29" t="inlineStr"/>
+      <c r="H9" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I9" s="29" t="inlineStr"/>
       <c r="J9" s="29" t="inlineStr"/>
       <c r="K9" s="29" t="inlineStr"/>
@@ -1947,7 +1963,11 @@
       <c r="E10" s="29" t="inlineStr"/>
       <c r="F10" s="29" t="inlineStr"/>
       <c r="G10" s="29" t="inlineStr"/>
-      <c r="H10" s="29" t="inlineStr"/>
+      <c r="H10" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I10" s="29" t="inlineStr"/>
       <c r="J10" s="29" t="inlineStr"/>
       <c r="K10" s="29" t="inlineStr"/>
@@ -1988,7 +2008,11 @@
       <c r="E11" s="29" t="inlineStr"/>
       <c r="F11" s="29" t="inlineStr"/>
       <c r="G11" s="29" t="inlineStr"/>
-      <c r="H11" s="29" t="inlineStr"/>
+      <c r="H11" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I11" s="29" t="inlineStr"/>
       <c r="J11" s="29" t="inlineStr"/>
       <c r="K11" s="29" t="inlineStr"/>
@@ -2091,7 +2115,11 @@
       <c r="E14" s="44" t="inlineStr"/>
       <c r="F14" s="44" t="inlineStr"/>
       <c r="G14" s="44" t="inlineStr"/>
-      <c r="H14" s="44" t="inlineStr"/>
+      <c r="H14" s="46" t="inlineStr">
+        <is>
+          <t>นพดล สุระแสน</t>
+        </is>
+      </c>
       <c r="I14" s="44" t="inlineStr"/>
       <c r="J14" s="44" t="inlineStr"/>
       <c r="K14" s="44" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for Crane no.2 Day 7
</commit_message>
<xml_diff>
--- a/FM-MN-07_Crane no.2.xlsx
+++ b/FM-MN-07_Crane no.2.xlsx
@@ -1789,7 +1789,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I6" s="29" t="inlineStr"/>
+      <c r="I6" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J6" s="29" t="inlineStr"/>
       <c r="K6" s="29" t="inlineStr"/>
       <c r="L6" s="29" t="inlineStr"/>
@@ -1834,7 +1838,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I7" s="29" t="inlineStr"/>
+      <c r="I7" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J7" s="29" t="inlineStr"/>
       <c r="K7" s="29" t="inlineStr"/>
       <c r="L7" s="29" t="inlineStr"/>
@@ -1880,7 +1888,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I8" s="29" t="inlineStr"/>
+      <c r="I8" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J8" s="29" t="inlineStr"/>
       <c r="K8" s="29" t="inlineStr"/>
       <c r="L8" s="29" t="inlineStr"/>
@@ -1925,7 +1937,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I9" s="29" t="inlineStr"/>
+      <c r="I9" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J9" s="29" t="inlineStr"/>
       <c r="K9" s="29" t="inlineStr"/>
       <c r="L9" s="29" t="inlineStr"/>
@@ -1971,7 +1987,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I10" s="29" t="inlineStr"/>
+      <c r="I10" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J10" s="29" t="inlineStr"/>
       <c r="K10" s="29" t="inlineStr"/>
       <c r="L10" s="29" t="inlineStr"/>
@@ -2016,7 +2036,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I11" s="29" t="inlineStr"/>
+      <c r="I11" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J11" s="29" t="inlineStr"/>
       <c r="K11" s="29" t="inlineStr"/>
       <c r="L11" s="29" t="inlineStr"/>
@@ -2123,7 +2147,11 @@
           <t>นพดล สุระแสน</t>
         </is>
       </c>
-      <c r="I14" s="44" t="inlineStr"/>
+      <c r="I14" s="46" t="inlineStr">
+        <is>
+          <t>นพดล สุระแสน</t>
+        </is>
+      </c>
       <c r="J14" s="44" t="inlineStr"/>
       <c r="K14" s="44" t="inlineStr"/>
       <c r="L14" s="44" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for Crane no.2 Day 8
</commit_message>
<xml_diff>
--- a/FM-MN-07_Crane no.2.xlsx
+++ b/FM-MN-07_Crane no.2.xlsx
@@ -1794,7 +1794,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J6" s="29" t="inlineStr"/>
+      <c r="J6" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K6" s="29" t="inlineStr"/>
       <c r="L6" s="29" t="inlineStr"/>
       <c r="M6" s="29" t="inlineStr"/>
@@ -1843,7 +1847,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J7" s="29" t="inlineStr"/>
+      <c r="J7" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K7" s="29" t="inlineStr"/>
       <c r="L7" s="29" t="inlineStr"/>
       <c r="M7" s="29" t="inlineStr"/>
@@ -1893,7 +1901,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J8" s="29" t="inlineStr"/>
+      <c r="J8" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K8" s="29" t="inlineStr"/>
       <c r="L8" s="29" t="inlineStr"/>
       <c r="M8" s="29" t="inlineStr"/>
@@ -1942,7 +1954,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J9" s="29" t="inlineStr"/>
+      <c r="J9" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K9" s="29" t="inlineStr"/>
       <c r="L9" s="29" t="inlineStr"/>
       <c r="M9" s="29" t="inlineStr"/>
@@ -1992,7 +2008,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J10" s="29" t="inlineStr"/>
+      <c r="J10" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K10" s="29" t="inlineStr"/>
       <c r="L10" s="29" t="inlineStr"/>
       <c r="M10" s="29" t="inlineStr"/>
@@ -2041,7 +2061,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J11" s="29" t="inlineStr"/>
+      <c r="J11" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K11" s="29" t="inlineStr"/>
       <c r="L11" s="29" t="inlineStr"/>
       <c r="M11" s="29" t="inlineStr"/>
@@ -2152,7 +2176,11 @@
           <t>นพดล สุระแสน</t>
         </is>
       </c>
-      <c r="J14" s="44" t="inlineStr"/>
+      <c r="J14" s="46" t="inlineStr">
+        <is>
+          <t>นพดล สุระแสน</t>
+        </is>
+      </c>
       <c r="K14" s="44" t="inlineStr"/>
       <c r="L14" s="44" t="inlineStr"/>
       <c r="M14" s="44" t="inlineStr"/>

</xml_diff>